<commit_message>
Sync complete pipeline, input files and results
</commit_message>
<xml_diff>
--- a/Data/Results/Data_Cleaning_Audit.xlsx
+++ b/Data/Results/Data_Cleaning_Audit.xlsx
@@ -14,8 +14,8 @@
     <sheet name="Cleaning Rules" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'File Summary'!$A$1:$M$35</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Removed Rows'!$A$1:$M$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'File Summary'!$A$1:$M$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Removed Rows'!$A$1:$M$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Speed Audit'!$A$1:$N$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Cleaning Rules'!$A$1:$F$13</definedName>
   </definedNames>
@@ -482,7 +482,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46294.46676650071</v>
+        <v>46301.96813307998</v>
       </c>
     </row>
     <row r="3">
@@ -516,7 +516,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>34</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6">
@@ -526,7 +526,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>34</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7">
@@ -556,7 +556,7 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>68274</v>
+        <v>80689</v>
       </c>
     </row>
     <row r="10">
@@ -576,7 +576,7 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12">
@@ -586,7 +586,7 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13">
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>68257</v>
+        <v>80668</v>
       </c>
     </row>
   </sheetData>
@@ -630,7 +630,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M35"/>
+  <dimension ref="A1:M41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -2016,7 +2016,7 @@
         </is>
       </c>
       <c r="F28" s="2" t="n">
-        <v>1259</v>
+        <v>1257</v>
       </c>
       <c r="G28" s="2" t="n">
         <v>0</v>
@@ -2034,7 +2034,7 @@
         <v>0</v>
       </c>
       <c r="L28" s="2" t="n">
-        <v>1259</v>
+        <v>1257</v>
       </c>
       <c r="M28" s="2" t="inlineStr"/>
     </row>
@@ -2286,12 +2286,12 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>chennai_to_pondicherry_ev_intercity.xlsx</t>
+          <t>chennai_to_pondicherry_diesel_intercity.xlsx</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>D:\Hameeda_Projects\TAT_MS_INTERCITY\Data\Input\25-09-2026\chennai_to_pondicherry_ev_intercity.xlsx</t>
+          <t>D:\Hameeda_Projects\TAT_MS_INTERCITY\Data\Input\25-09-2026\chennai_to_pondicherry_diesel_intercity.xlsx</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -2310,7 +2310,7 @@
         </is>
       </c>
       <c r="F34" s="2" t="n">
-        <v>2584</v>
+        <v>958</v>
       </c>
       <c r="G34" s="2" t="n">
         <v>0</v>
@@ -2322,67 +2322,361 @@
         <v>0</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L34" s="2" t="n">
-        <v>2584</v>
+        <v>957</v>
       </c>
       <c r="M34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
+          <t>chennai_to_pondicherry_ev_intercity.xlsx</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>D:\Hameeda_Projects\TAT_MS_INTERCITY\Data\Input\25-09-2026\chennai_to_pondicherry_ev_intercity.xlsx</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>DEVICE_RAW</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Sheet1</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>CLEANED</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="n">
+        <v>2584</v>
+      </c>
+      <c r="G35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" s="2" t="n">
+        <v>2584</v>
+      </c>
+      <c r="M35" s="2" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>pondicherry_to_chennai_diesel_intercity.xlsx</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>D:\Hameeda_Projects\TAT_MS_INTERCITY\Data\Input\26-09-2026\pondicherry_to_chennai_diesel_intercity.xlsx</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>DEVICE_RAW</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Sheet1</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>CLEANED</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="n">
+        <v>973</v>
+      </c>
+      <c r="G36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L36" s="2" t="n">
+        <v>973</v>
+      </c>
+      <c r="M36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
           <t>pondicherry_to_chennai_ev_intercity.xlsx</t>
         </is>
       </c>
-      <c r="B35" s="2" t="inlineStr">
+      <c r="B37" s="2" t="inlineStr">
         <is>
           <t>D:\Hameeda_Projects\TAT_MS_INTERCITY\Data\Input\26-09-2026\pondicherry_to_chennai_ev_intercity.xlsx</t>
         </is>
       </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>DEVICE_RAW</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>Sheet1</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>DEVICE_RAW</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Sheet1</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
         <is>
           <t>CLEANED</t>
         </is>
       </c>
-      <c r="F35" s="2" t="n">
+      <c r="F37" s="2" t="n">
         <v>2675</v>
       </c>
-      <c r="G35" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H35" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I35" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J35" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K35" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L35" s="2" t="n">
+      <c r="G37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L37" s="2" t="n">
         <v>2675</v>
       </c>
-      <c r="M35" s="2" t="inlineStr"/>
+      <c r="M37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>maduravoyal_to_madiwala_diesel_intercity.xlsx</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>D:\Hameeda_Projects\TAT_MS_INTERCITY\Data\Input\02-10-2026\maduravoyal_to_madiwala_diesel_intercity.xlsx</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>DEVICE_RAW</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Sheet1</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>CLEANED</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="n">
+        <v>1344</v>
+      </c>
+      <c r="G38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J38" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K38" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="L38" s="2" t="n">
+        <v>1342</v>
+      </c>
+      <c r="M38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>maduravoyal_to_madiwala_ev_intercity.xlsx</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>D:\Hameeda_Projects\TAT_MS_INTERCITY\Data\Input\02-10-2026\maduravoyal_to_madiwala_ev_intercity.xlsx</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>DEVICE_RAW</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Sheet1</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>CLEANED</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="n">
+        <v>3632</v>
+      </c>
+      <c r="G39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J39" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K39" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L39" s="2" t="n">
+        <v>3631</v>
+      </c>
+      <c r="M39" s="2" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>madiwala_to_maduravoyal_diesel_intercity.xlsx</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>D:\Hameeda_Projects\TAT_MS_INTERCITY\Data\Input\03-10-2026\madiwala_to_maduravoyal_diesel_intercity.xlsx</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>DEVICE_RAW</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Sheet1</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>CLEANED</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="n">
+        <v>1273</v>
+      </c>
+      <c r="G40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L40" s="2" t="n">
+        <v>1273</v>
+      </c>
+      <c r="M40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>madiwala_to_maduravoyal_ev_intercity.xlsx</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>D:\Hameeda_Projects\TAT_MS_INTERCITY\Data\Input\03-10-2026\madiwala_to_maduravoyal_ev_intercity.xlsx</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>DEVICE_RAW</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Sheet1</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>CLEANED</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="n">
+        <v>4237</v>
+      </c>
+      <c r="G41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L41" s="2" t="n">
+        <v>4237</v>
+      </c>
+      <c r="M41" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M35"/>
+  <autoFilter ref="A1:M41"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2393,7 +2687,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M18"/>
+  <dimension ref="A1:M22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -3413,8 +3707,228 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>chennai_to_pondicherry_diesel_intercity.xlsx</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>D:\Hameeda_Projects\TAT_MS_INTERCITY\Data\Input\25-09-2026\chennai_to_pondicherry_diesel_intercity.xlsx</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>DEVICE_RAW</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Sheet1</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>949</v>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>DUPLICATE_REMOVAL</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Exact duplicate of an earlier standardized telemetry row; first occurrence retained</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="n">
+        <v>46290.81975694445</v>
+      </c>
+      <c r="I19" s="2" t="n">
+        <v>11.93717</v>
+      </c>
+      <c r="J19" s="2" t="n">
+        <v>79.81885</v>
+      </c>
+      <c r="K19" s="2" t="n">
+        <v>1.111111111111111</v>
+      </c>
+      <c r="L19" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>Thiruvalluvar Road, Sithankudi, Oulgaret, Ozhukarai Taluk, Brindavanam, Puducherry, 605013, India</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>maduravoyal_to_madiwala_diesel_intercity.xlsx</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>D:\Hameeda_Projects\TAT_MS_INTERCITY\Data\Input\02-10-2026\maduravoyal_to_madiwala_diesel_intercity.xlsx</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>DEVICE_RAW</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Sheet1</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>1157</v>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>DUPLICATE_REMOVAL</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Exact duplicate of an earlier standardized telemetry row; first occurrence retained</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="n">
+        <v>46298.17877314815</v>
+      </c>
+      <c r="I20" s="2" t="n">
+        <v>12.77718</v>
+      </c>
+      <c r="J20" s="2" t="n">
+        <v>77.77607</v>
+      </c>
+      <c r="K20" s="2" t="n">
+        <v>1.111111111111111</v>
+      </c>
+      <c r="L20" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>Chennekothapalli Rd, Attibele, Karnataka 562107, India</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>maduravoyal_to_madiwala_diesel_intercity.xlsx</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>D:\Hameeda_Projects\TAT_MS_INTERCITY\Data\Input\02-10-2026\maduravoyal_to_madiwala_diesel_intercity.xlsx</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>DEVICE_RAW</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Sheet1</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>1344</v>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>DUPLICATE_REMOVAL</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Exact duplicate of an earlier standardized telemetry row; first occurrence retained</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="n">
+        <v>46298.22202546296</v>
+      </c>
+      <c r="I21" s="2" t="n">
+        <v>12.96495</v>
+      </c>
+      <c r="J21" s="2" t="n">
+        <v>77.59851999999999</v>
+      </c>
+      <c r="K21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>Thales, Richmond Road, Langford Gardens, Bengaluru, Bangalore North, Richmond Town, Karnataka, 560001, India</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>maduravoyal_to_madiwala_ev_intercity.xlsx</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>D:\Hameeda_Projects\TAT_MS_INTERCITY\Data\Input\02-10-2026\maduravoyal_to_madiwala_ev_intercity.xlsx</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>DEVICE_RAW</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Sheet1</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>2769</v>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>DUPLICATE_REMOVAL</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Exact duplicate of an earlier standardized telemetry row; first occurrence retained</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="n">
+        <v>46298.17090277778</v>
+      </c>
+      <c r="I22" s="2" t="n">
+        <v>12.6264</v>
+      </c>
+      <c r="J22" s="2" t="n">
+        <v>78.07932</v>
+      </c>
+      <c r="K22" s="2" t="n">
+        <v>16.66666666666667</v>
+      </c>
+      <c r="L22" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>Chennekothapalli Rd, Mallasandiram, Tamil Nadu 635117, India</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M18"/>
+  <autoFilter ref="A1:M22"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>